<commit_message>
Editor de diseño de hojas + hoja Diapositivas
</commit_message>
<xml_diff>
--- a/data/informe.xlsx
+++ b/data/informe.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acciones_Rehabilitacion" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seguimiento_Contactabilidad" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insumo_Sujetos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diapositivas" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -81,13 +82,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3675,4 +3679,660 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Seccion</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Orden</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Activa</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Bloque</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Celda</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Contenido</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Cifra</t>
+        </is>
+      </c>
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Fondo</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>Imagen</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
+          <t>Ajuste</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Resumen del corte</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Lectura del corte</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>El avance del mes se concentró en las medidas de rehabilitación de los resguardos de Risaralda y el cierre de encuentros GAM con el grupo de periodistas en Nariño. Las tres entregas de maquinaria amarilla continúan en etapa de importación.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>blanco</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Resumen del corte</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>acciones implementadas al corte</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>azul</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Resumen del corte</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>de contactabilidad efectiva</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>74.4%</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>dorado</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Resumen del corte</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>acciones pendientes por trámites</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>rojo</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Resumen del corte</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>departamentos con implementación</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>gris</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Sujetos con maquinaria amarilla</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>tabla</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Maquinaria_Amarilla</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sujetos con documentación completa</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>tabla</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Documentacion_Completa</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="n"/>
+      <c r="N8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sujetos con acompañamiento para envío de la documentación</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>tabla</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Acompanamiento_Documentacion</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Acciones rehabilitación</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>tabla</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Acciones_Rehabilitacion</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Seguimiento de Contactabilidad</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>contactabilidad</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Mapa de implementación por departamento</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>mapa</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n"/>
+      <c r="K12" s="2" t="n"/>
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Jornada destacada — Telar Luz del Amanecer</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>imagen+texto</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Telar Luz del Amanecer</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Día de conmemoración por las víctimas del colectivo — Valle del Guamuez, Putumayo.</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>blanco</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Luz_Telar_2.jpeg</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>recortar</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Jornada destacada — Telar Luz del Amanecer</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>imagen</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>blanco</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Luz_Telar_7.jpeg</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>recortar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Token persistente en el equipo
</commit_message>
<xml_diff>
--- a/data/informe.xlsx
+++ b/data/informe.xlsx
@@ -3687,92 +3687,98 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
+          <t>Hoja</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
           <t>Seccion</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Orden</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Activa</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Fuente</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Bloque</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Celda</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Contenido</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Titulo</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Detalle</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Cifra</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Fondo</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Imagen</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Ajuste</t>
         </is>
@@ -3781,440 +3787,502 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Resumen del corte</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
+          <t>Portada</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>bloques</t>
-        </is>
-      </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>campo</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>texto</t>
-        </is>
-      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Lectura del corte</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>El avance del mes se concentró en las medidas de rehabilitación de los resguardos de Risaralda y el cierre de encuentros GAM con el grupo de periodistas en Nariño. Las tres entregas de maquinaria amarilla continúan en etapa de importación.</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>blanco</t>
-        </is>
-      </c>
+          <t>eyebrow</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Convenio 3007 de 2025</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Resumen del corte</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>bloques</t>
-        </is>
+          <t>Portada</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>campo</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>texto</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>acciones implementadas al corte</t>
-        </is>
-      </c>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>azul</t>
-        </is>
-      </c>
+          <t>Informe de Seguimiento</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Resumen del corte</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>bloques</t>
-        </is>
+          <t>Portada</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>campo</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>texto</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>de contactabilidad efectiva</t>
-        </is>
-      </c>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>subtitulo</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>74.4%</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>dorado</t>
-        </is>
-      </c>
+          <t>Análisis de Ejecución y Contactabilidad</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="n"/>
       <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Resumen del corte</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>bloques</t>
-        </is>
+          <t>Portada</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>campo</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G5" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>texto</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>acciones pendientes por trámites</t>
-        </is>
-      </c>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>etiqueta</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>rojo</t>
-        </is>
-      </c>
+          <t>Implementación de Planes Integrales de Reparación Colectiva</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="n"/>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="n"/>
+      <c r="O5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Resumen del corte</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>bloques</t>
-        </is>
+          <t>Portada</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>campo</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>texto</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>departamentos con implementación</t>
-        </is>
-      </c>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>convenio</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>gris</t>
-        </is>
-      </c>
+          <t>Convenio 3007 de 2025</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="n"/>
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="n"/>
+      <c r="O6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Sujetos con maquinaria amarilla</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>tabla</t>
-        </is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Resumen del corte</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Maquinaria_Amarilla</t>
-        </is>
-      </c>
       <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
+      <c r="G7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Lectura del corte</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>El avance del mes se concentró en las medidas de rehabilitación de los resguardos de Risaralda y el cierre de encuentros GAM con el grupo de periodistas en Nariño. Las tres entregas de maquinaria amarilla continúan en etapa de importación.</t>
+        </is>
+      </c>
       <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>blanco</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Sujetos con documentación completa</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>tabla</t>
-        </is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Resumen del corte</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Documentacion_Completa</t>
-        </is>
-      </c>
       <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
+      <c r="G8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
       <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="n"/>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>acciones implementadas al corte</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>azul</t>
+        </is>
+      </c>
       <c r="N8" s="2" t="n"/>
+      <c r="O8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Sujetos con acompañamiento para envío de la documentación</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>tabla</t>
-        </is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Resumen del corte</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Acompanamiento_Documentacion</t>
-        </is>
-      </c>
       <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
+      <c r="G9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="n"/>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>de contactabilidad efectiva</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>74.4%</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>dorado</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Acciones rehabilitación</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>tabla</t>
-        </is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Resumen del corte</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Acciones_Rehabilitacion</t>
-        </is>
-      </c>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
+      <c r="G10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>acciones pendientes por trámites</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>rojo</t>
+        </is>
+      </c>
       <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Seguimiento de Contactabilidad</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>contactabilidad</t>
-        </is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Resumen del corte</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
-      <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="n"/>
+      <c r="G11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>departamentos con implementación</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>gris</t>
+        </is>
+      </c>
       <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Mapa de implementación por departamento</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>mapa</t>
-        </is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Sujetos con maquinaria amarilla</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>tabla</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Maquinaria_Amarilla</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="n"/>
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
@@ -4223,114 +4291,605 @@
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Jornada destacada — Telar Luz del Amanecer</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>bloques</t>
-        </is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Sujetos con documentación completa</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>tabla</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>imagen+texto</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Telar Luz del Amanecer</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Día de conmemoración por las víctimas del colectivo — Valle del Guamuez, Putumayo.</t>
-        </is>
-      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Documentacion_Completa</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>blanco</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>Luz_Telar_2.jpeg</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>recortar</t>
-        </is>
-      </c>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Jornada destacada — Telar Luz del Amanecer</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>bloques</t>
-        </is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Sujetos con acompañamiento para envío de la documentación</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>tabla</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>imagen</t>
-        </is>
-      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Acompanamiento_Documentacion</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Acciones rehabilitación</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>tabla</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Acciones_Rehabilitacion</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n"/>
+      <c r="M15" s="2" t="n"/>
+      <c r="N15" s="2" t="n"/>
+      <c r="O15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Seguimiento de Contactabilidad</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>contactabilidad</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n"/>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Mapa de implementación por departamento</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>mapa</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="2" t="n"/>
+      <c r="O17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Jornada destacada — Telar Luz del Amanecer</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>imagen+texto</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Telar Luz del Amanecer</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Día de conmemoración por las víctimas del colectivo — Valle del Guamuez, Putumayo.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="n"/>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>blanco</t>
         </is>
       </c>
-      <c r="M14" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Luz_Telar_2.jpeg</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>recortar</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Informe</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Jornada destacada — Telar Luz del Amanecer</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>imagen</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>blanco</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>Luz_Telar_7.jpeg</t>
         </is>
       </c>
-      <c r="N14" s="2" t="inlineStr">
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>recortar</t>
         </is>
       </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Caso 1</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Consejo Comunitario Flamenco</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>hoja</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n"/>
+      <c r="K20" s="2" t="n"/>
+      <c r="L20" s="2" t="n"/>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="2" t="n"/>
+      <c r="O20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Caso 1</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Contexto del caso</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>imagen+texto</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Comunidad Afrodescendiente Flamenco</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>María La Baja, Bolívar. Avanza la medida de rehabilitación con las tertulias de trámite del dolor, sanación y armonía espiritual dirigidas a las mujeres del colectivo.</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="n"/>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>blanco</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Flamenco_1.jpeg</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>recortar</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Caso 1</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Contexto del caso</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>bloques</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Estado de la acción</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Primera de tres tertulias realizada; las dos restantes están programadas para el tercer trimestre, con proyección de costos de $ 9.475.574.</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>gris</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n"/>
+      <c r="O22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Caso 2</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Caso 2</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>hoja</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="n"/>
+      <c r="N23" s="2" t="n"/>
+      <c r="O23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Caso 3</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Caso 3</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>hoja</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n"/>
+      <c r="K24" s="2" t="n"/>
+      <c r="L24" s="2" t="n"/>
+      <c r="M24" s="2" t="n"/>
+      <c r="N24" s="2" t="n"/>
+      <c r="O24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Caso 4</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Caso 4</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>hoja</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
+      <c r="I25" s="2" t="n"/>
+      <c r="J25" s="2" t="n"/>
+      <c r="K25" s="2" t="n"/>
+      <c r="L25" s="2" t="n"/>
+      <c r="M25" s="2" t="n"/>
+      <c r="N25" s="2" t="n"/>
+      <c r="O25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Caso 5</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Caso 5</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>hoja</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="n"/>
+      <c r="K26" s="2" t="n"/>
+      <c r="L26" s="2" t="n"/>
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2" t="n"/>
+      <c r="O26" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Actualización de diseño desde el informe interactivo
</commit_message>
<xml_diff>
--- a/data/informe.xlsx
+++ b/data/informe.xlsx
@@ -405,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -426,12 +426,6 @@
       <c r="F1" t="str">
         <v>Actividad / Accion</v>
       </c>
-      <c r="G1" t="str">
-        <v>Proyeccion de costos</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Observaciones</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -452,12 +446,6 @@
       <c r="F2" t="str">
         <v>Realizar la entrega del banco de maquinaria</v>
       </c>
-      <c r="G2">
-        <v>3017488000</v>
-      </c>
-      <c r="H2" t="str">
-        <v>El proceso de importacion tiene un tiempo entre 1 a 3 meses.</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -478,9 +466,6 @@
       <c r="F3" t="str">
         <v>Entrega de un Banco de maquinaria amarilla compuesto por una retroexcavadora pajarita, una volqueta y una motoniveladora.</v>
       </c>
-      <c r="H3" t="str">
-        <v>Pendiente de costeo - falta numero de accion asignado.</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -501,24 +486,18 @@
       <c r="F4" t="str">
         <v>4. Entrega maquinaria amarilla</v>
       </c>
-      <c r="G4">
-        <v>792070436</v>
-      </c>
-      <c r="H4" t="str">
-        <v>El proceso de importacion tiene un tiempo entre 1 a 3 meses.</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:E16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -528,140 +507,274 @@
         <v>Caso Nombre</v>
       </c>
       <c r="C1" t="str">
-        <v>Medida ID</v>
+        <v>Accion ID</v>
       </c>
       <c r="D1" t="str">
-        <v>Producto / Medida</v>
+        <v>Actividad / Accion</v>
       </c>
       <c r="E1" t="str">
-        <v>Accion ID</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Actividad / Accion</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Proyeccion de costos</v>
+        <v>profesional acopaña</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ordenes Judiciales</v>
+        <v>Ordenes judiciales</v>
       </c>
       <c r="B2" t="str">
-        <v>557 - CONSEJO COMUNITARIO RIO TABLON DULCE</v>
+        <v>252 - CONSEJO COMUNITARIO RIO LA LARGA Y TUMARADO (COCOLATU)</v>
       </c>
       <c r="C2">
-        <v>44992</v>
+        <v>39472</v>
       </c>
       <c r="D2" t="str">
-        <v>Servicios de realizacion de eventos relacionados con practicas tradicionales, sociales y culturales afectadas por el conflicto armado</v>
-      </c>
-      <c r="E2">
-        <v>45040</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Realizar la fiesta patronal del 20 de enero en honor de San Sebastian.</v>
-      </c>
-      <c r="G2">
-        <v>127308000</v>
+        <v>Realizar el requerimiento de intervenciones menores para la construcción del mural de la memoria</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Andrea Garcia</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Ordenes Judiciales</v>
+        <v>Ordenes judiciales</v>
       </c>
       <c r="B3" t="str">
-        <v>404 - CONSEJO COMUNITARIO AIRES DE GARRAPATERO</v>
+        <v>252 - CONSEJO COMUNITARIO RIO LA LARGA Y TUMARADO (COCOLATU)</v>
       </c>
       <c r="C3">
-        <v>35264</v>
+        <v>39473</v>
       </c>
       <c r="D3" t="str">
-        <v>Infraestructura de produccion agricola adecuada</v>
-      </c>
-      <c r="E3">
-        <v>35267</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Realizar la compra de los materiales de construccion requeridos para la adecuacion del trapiche comunitario</v>
-      </c>
-      <c r="G3">
-        <v>99670404.96</v>
+        <v>Realizar la entrega de los materiales para la construcción del mural de la me...</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Andrea Garcia</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Ordenes Judiciales</v>
+        <v>Ordenes judiciales</v>
       </c>
       <c r="B4" t="str">
-        <v>243 - PUEBLO KANKUAMO</v>
+        <v>252 - CONSEJO COMUNITARIO RIO LA LARGA Y TUMARADO (COCOLATU)</v>
       </c>
       <c r="C4">
-        <v>50303</v>
+        <v>39474</v>
       </c>
       <c r="D4" t="str">
-        <v>Centros comunitarios adecuados</v>
-      </c>
-      <c r="E4">
-        <v>50346</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Construir seis kankuruas ubicadas en las comunidades de Ramatio, Mojao y Rancho de la Goya - Resguardo Indigena Kankuamo.</v>
-      </c>
-      <c r="G4">
-        <v>875869616</v>
+        <v>Realizar la demarcación en el cementerio como un lugar de memoria</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Andrea Garcia</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Ordenes Judiciales</v>
+        <v>Ordenes judiciales</v>
       </c>
       <c r="B5" t="str">
-        <v>706 - CABILDO INDIGENA TELAR LUZ DEL AMANECER</v>
+        <v>252 - CONSEJO COMUNITARIO RIO LA LARGA Y TUMARADO (COCOLATU)</v>
       </c>
       <c r="C5">
-        <v>49441</v>
+        <v>39475</v>
       </c>
       <c r="D5" t="str">
-        <v>Actos simbolicos y de dignificacion</v>
-      </c>
-      <c r="E5">
-        <v>49452</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Realizar el Dia de conmemoracion por las victimas del colectivo</v>
-      </c>
-      <c r="G5">
-        <v>59234643</v>
+        <v>Realizar el seguimiento al producto de servicios de demarcación de lugares de...</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Andrea Garcia</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>Ordenes judiciales</v>
+      </c>
+      <c r="B6" t="str">
+        <v>557 - CONSEJO COMUNITARIO RIO TABLON DULCE. NARIÑO -TUMACO</v>
+      </c>
+      <c r="C6">
+        <v>45040</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Realizar la fiesta patronal del 20 de enero en honor de San Sebastián.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Daniel Marin</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Ordenes judiciales</v>
+      </c>
+      <c r="B7" t="str">
+        <v>650 - RESGUARDO INDIGENA LA ARGELIA - PUTUMAYO</v>
+      </c>
+      <c r="C7">
+        <v>42782</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Recopilar la información para la , diagramación e impresión de 300 cartillas</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Imelda Perez</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Ordenes judiciales</v>
+      </c>
+      <c r="B8" t="str">
+        <v>706 - CABILDO INDÍGENA TELAR LUZ DEL AMANECER - PUTUMAYO</v>
+      </c>
+      <c r="C8">
+        <v>49451</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Realizar una jornada preparatoria para el desarrollo del acto de conmemoración</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Imelda Perez</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Ordenes judiciales</v>
+      </c>
+      <c r="B9" t="str">
+        <v>706 - CABILDO INDÍGENA TELAR LUZ DEL AMANECER - PUTUMAYO</v>
+      </c>
+      <c r="C9">
+        <v>49452</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Realizar el Día de conmemoración por las víctimas del colectivo</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Imelda Perez</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>acciones no implementada.</v>
+      </c>
+      <c r="B10" t="str">
+        <v>774 - CHITACOYDCABILDO INDIGENA HEREDEROS DE TABACO ,COCA Y YUCA DULCE</v>
+      </c>
+      <c r="C10">
+        <v>33795</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Apoyar la revitalización delplan de vida.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Lizeth Castillo</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>fase de ruta</v>
+      </c>
+      <c r="B11" t="str">
+        <v>986 - RESGUARDO LA SORTIJA - TOLIMA (ORTEGA)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Fase de ruta / caracterización del daño</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Implementación de la acción para la jornada de caracterización del daño del Resguardo Indígena La Sortija.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Lizeth Castillo</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>Ordenes Judiciales</v>
       </c>
-      <c r="B6" t="str">
-        <v>706 - CABILDO INDIGENA TELAR LUZ DEL AMANECER</v>
-      </c>
-      <c r="C6">
-        <v>49449</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Servicio de apoyo a las formas propias de proteccion comunitaria y control territorial etnicas</v>
-      </c>
-      <c r="E6">
-        <v>49491</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Realizar taller de capacitacion a la guardia indigena</v>
-      </c>
-      <c r="G6">
-        <v>59234643</v>
+      <c r="B12" t="str">
+        <v>86 - RESGUARDO EMBERA LOMA CITABARA</v>
+      </c>
+      <c r="C12">
+        <v>42978</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Espacios de formación  sobre las prácticas médicas y  ancestrales a las comunidades</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Imelda Perez</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Ordenes Judiciales</v>
+      </c>
+      <c r="B13" t="str">
+        <v>88 - RESGUARDO GITO DOKABU</v>
+      </c>
+      <c r="C13">
+        <v>43555</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Realizar ceremonia espiritual y ritual de limpieza en las comunidades de Canchido y cuna Gito</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Lina Londoño</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Ordenes Judiciales</v>
+      </c>
+      <c r="B14" t="str">
+        <v>88 - RESGUARDO GITO DOKABU</v>
+      </c>
+      <c r="C14">
+        <v>43556</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Realizar ceremonia espiritual y ritual de limpieza en las comunidades de Buenos Aires y Playitas</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Lina Londoño</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>acciones no implementada.</v>
+      </c>
+      <c r="B15" t="str">
+        <v>317 - PERIODISTA CORPORACION  VICTIMAS DEL CONFLICTO ARMADO DE COLOMBIA</v>
+      </c>
+      <c r="C15">
+        <v>38778</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Realizar los 4 encuentros del GAM con el tercer grupo de periodistas</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Lina Londoño</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>acciones no implementada.</v>
+      </c>
+      <c r="B16" t="str">
+        <v>501 - FLAMENCO CONSEJO COMUNITARIO DE COMUNIDADES NEGRAS. MARIA L ABAJA</v>
+      </c>
+      <c r="C16">
+        <v>48558</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Realizar un encuentro para tramite del dolo con el grupo de oración de flamenco</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Lina Londoño</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>